<commit_message>
feat(masterdata): KnockbackEffect bean 추가 (write_beans_index + __beans__ 재생성)
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/table/Datas/__beans__.xlsx
+++ b/table/Datas/__beans__.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P8"/>
+  <dimension ref="A1:P13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -702,6 +702,148 @@
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr"/>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr"/>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>KnockbackEffect</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>AbilityEffect</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>넉백 — 공격자 반대로 밀기(지수 감쇠)</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>strength</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr"/>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>range</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr"/>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>angle</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr"/>
+      <c r="B12" t="inlineStr"/>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>duration_ticks</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr"/>
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>decay_per_tick</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="J1:P1"/>

</xml_diff>

<commit_message>
chore(masterdata): 넉백 KnockbackEffect Range/Angle 잔재 제거 (Luban 소스)
Part 1에서 히트 형상이 데미지 효과로 이관되며 넉백엔 미사용으로 남은
range/angle을 KnockbackEffect bean(__beans__.xlsx)과 attack 데이터(#Ability.xlsx)에서 제거.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/table/Datas/__beans__.xlsx
+++ b/table/Datas/__beans__.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P13"/>
+  <dimension ref="A1:P11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -474,14 +474,6 @@
           <t>##var</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr">
         <is>
           <t>name</t>
@@ -519,33 +511,18 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr"/>
       <c r="B3" t="inlineStr">
         <is>
           <t>AbilityEffect</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>polymorphic base</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr"/>
       <c r="B4" t="inlineStr">
         <is>
           <t>StatusEffectApplyEffect</t>
@@ -556,30 +533,18 @@
           <t>AbilityEffect</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr">
         <is>
           <t>status_effect_id</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr">
         <is>
           <t>int</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
           <t>MotionEffect</t>
@@ -590,30 +555,18 @@
           <t>AbilityEffect</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr">
         <is>
           <t>speed</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr">
         <is>
           <t>float</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr">
         <is>
           <t>DamageEffect</t>
@@ -624,86 +577,47 @@
           <t>AbilityEffect</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
           <t>데미지 + 부채꼴 타게팅 형상</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr">
         <is>
           <t>amount</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
           <t>int</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr"/>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr">
         <is>
           <t>range</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr">
         <is>
           <t>float</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr"/>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr">
         <is>
           <t>angle</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
           <t>float</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr"/>
       <c r="B9" t="inlineStr">
         <is>
           <t>KnockbackEffect</t>
@@ -714,135 +628,45 @@
           <t>AbilityEffect</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
           <t>넉백 — 공격자 반대로 밀기(지수 감쇠)</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr">
         <is>
           <t>strength</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
           <t>float</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
-      <c r="P9" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr"/>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr">
         <is>
-          <t>range</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr"/>
+          <t>duration_ticks</t>
+        </is>
+      </c>
       <c r="L10" t="inlineStr">
         <is>
+          <t>int</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>decay_per_tick</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
           <t>float</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr"/>
-      <c r="P10" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr"/>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>angle</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr"/>
-      <c r="P11" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr"/>
-      <c r="B12" t="inlineStr"/>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>duration_ticks</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>int</t>
-        </is>
-      </c>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr"/>
-      <c r="P12" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr"/>
-      <c r="B13" t="inlineStr"/>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>decay_per_tick</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr"/>
-      <c r="O13" t="inlineStr"/>
-      <c r="P13" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>